<commit_message>
Era-aware audit, srovnání schématu a propojení napříč 73 sezónami
- validate_almanach.py: era-aware audit → docs/DATA_QUALITY.md
  - mistr z META 'Mistr:' (pravý play-off vítěz) vs 1. místo ZČ; ≠ZČ u 30 sezón
  - 1949/50 vyřešeno: mistr = ATK Praha (1. místo), ne Zdar LTC (3.)
  - validace 2-1-0 (<2002) vs 3-2-1-0 (≥2002); moderní W/D/L ztrátový → neflaguje se
  - přesný seznam poškozených buněk: GA (1980/81,1981/82,2000/01,2001/02), GF (1991-95)
- harmonize_schema.py: SYSTEM srovnán na kanonických 12 sloupců (8 sezón doplněno)
- add_prev_node_id: prev_node_id doplněn i pro nové sezóny (propojení soutěží)
- apply_todo_sheets: nově flaguje poškozené GA/GF v TODO/NOTES; refresh všech 73
- health.py: 0 rozbitých prev linků, 0 fate nekonzistencí, 0 orphanů
- MASTER_REPORT + README aktualizovány (73 sezón, nové nástroje, stav nálezů)
- Pozn.: web-dohledání GA/GF nešlo (prostředí blokuje WebFetch); data se nevymýšlí, jen označují
</commit_message>
<xml_diff>
--- a/data/S1948_49_FINAL.xlsx
+++ b/data/S1948_49_FINAL.xlsx
@@ -1,21 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_liga" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KVAL" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SYSTEM" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CLUBS" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SERIES" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NOTES" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="META" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="10_liga" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="KVAL" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="SYSTEM" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="CLUBS" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="SERIES" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="NOTES" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="META" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="TODO" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'TODO'!$A$1:$F$2</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -23,7 +26,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -31,13 +34,22 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00305496"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -52,8 +64,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1509,7 +1527,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1541,6 +1559,36 @@
       <c r="F1" t="inlineStr">
         <is>
           <t>parent_node_id</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>feeds_into</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>feeds_into_loser</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>scoring</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>prev_node_id</t>
         </is>
       </c>
     </row>
@@ -2222,7 +2270,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:A4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2246,6 +2294,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2407,4 +2456,79 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="88" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>typ</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>reference</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>popis</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>vyřešeno? (ANO/ne)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>poznámka kolegy</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>pyramida (feeds_into)</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>NODE_S1948_49_0002</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>top-level kvalifikace bez feeds_into: 'Kvalifikace o ligu'</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F2"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Přidat sezónu 1947/48 z PDF + navázat chain na 1948/49 (DB: 73→74 sezón)
build_1947_48.py postavil S1947_48 (Státní liga: 2 skupiny po 6 + finále) z
sources/CZE1/CZ-1947-48.pdf. Ověřeno: sumy GF=GA (A 172, B 161), body=2V+R.
Mistr LTC Praha (finále 7:1, 13:5 nad I. ČLTK). Rozsah PARTIAL (jen nejvyšší
soutěž, jako 1948/49 — nižší/regiony později).

Navázáno 7 prev_club_id z 1948/49 na 1947/48 (LTC, ŠK Bratislava, Sparta Bubeneč,
Stadion ČB, Sokol Prostějov, I. ČLTK, Židenice<-Třebíč). DB nyní 74 sezón
(1947/48–2020/21), nejdelší řetěz 74 (LTC->...->Sparta), 0 rozbitých.
Starší 1946/47- zatím ne (chirurgická práce na později). README+MASTER_REPORT.
</commit_message>
<xml_diff>
--- a/data/S1948_49_FINAL.xlsx
+++ b/data/S1948_49_FINAL.xlsx
@@ -1775,9 +1775,14 @@
           <t>L10</t>
         </is>
       </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>CLUB_S1947_48_0007</t>
+        </is>
+      </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Republiková úroveň z Wiki (en). Prev_club_id nevyplněn (S1947_48 zatím nezpracována).</t>
+          <t>prev_club_id doplněn ze S1947_48 (nejvyšší soutěž z PDF).</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -1812,9 +1817,14 @@
           <t>L10</t>
         </is>
       </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>CLUB_S1947_48_0008</t>
+        </is>
+      </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Republiková úroveň z Wiki (en). Prev_club_id nevyplněn (S1947_48 zatím nezpracována).</t>
+          <t>prev_club_id doplněn ze S1947_48 (nejvyšší soutěž z PDF).</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -1886,9 +1896,14 @@
           <t>L10</t>
         </is>
       </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>CLUB_S1947_48_0010</t>
+        </is>
+      </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Republiková úroveň z Wiki (en). Prev_club_id nevyplněn (S1947_48 zatím nezpracována).</t>
+          <t>prev_club_id doplněn ze S1947_48 (nejvyšší soutěž z PDF).</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -1923,9 +1938,14 @@
           <t>L10</t>
         </is>
       </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>CLUB_S1947_48_0004</t>
+        </is>
+      </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Republiková úroveň z Wiki (en). Prev_club_id nevyplněn (S1947_48 zatím nezpracována).</t>
+          <t>prev_club_id doplněn ze S1947_48 (nejvyšší soutěž z PDF).</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -1960,9 +1980,14 @@
           <t>L10</t>
         </is>
       </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>CLUB_S1947_48_0009</t>
+        </is>
+      </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Republiková úroveň z Wiki (en). Prev_club_id nevyplněn (S1947_48 zatím nezpracována).</t>
+          <t>prev_club_id doplněn ze S1947_48 (nejvyšší soutěž z PDF).</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -1997,9 +2022,14 @@
           <t>L10</t>
         </is>
       </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>CLUB_S1947_48_0003</t>
+        </is>
+      </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Republiková úroveň z Wiki (en). Prev_club_id nevyplněn (S1947_48 zatím nezpracována).</t>
+          <t>prev_club_id doplněn ze S1947_48 (nejvyšší soutěž z PDF).</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -2034,9 +2064,14 @@
           <t>L10</t>
         </is>
       </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>CLUB_S1947_48_0001</t>
+        </is>
+      </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Republiková úroveň z Wiki (en). Prev_club_id nevyplněn (S1947_48 zatím nezpracována).</t>
+          <t>prev_club_id doplněn ze S1947_48 (nejvyšší soutěž z PDF).</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -2270,7 +2305,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A4"/>
+  <dimension ref="A1:A3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2294,7 +2329,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
1948/49: srovnat nejvyšší soutěž s PDF (sokolské názvy + poznámky) + Středočeská divize
enrich_1948_49.py (in-place):
- Státní liga: čísla už seděla; doplněny oficiální sokolské názvy do raw_name
  (JTO Sokol Pražský=LTC, ZJ Sokol NV Bratislava=ŠK Bratislava…), clean_name čitelný
  zůstává; věrné poznámky z PDF (sjednocení pod JTO Sokol 31.3.1948, sloučení
  Třebíč+Židenice 3.11., vyřazení Stadionu Podolí 9.11., stadiony).
- Středočeská divize (Skupina A+B) jako první nižší region: list 30STRC + SYSTEM
  uzly + 14 klubů. Ověřeno GF=GA (174:174, 289:289), body=2V+R.
</commit_message>
<xml_diff>
--- a/data/S1948_49_FINAL.xlsx
+++ b/data/S1948_49_FINAL.xlsx
@@ -15,6 +15,7 @@
     <sheet name="NOTES" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="META" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="TODO" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="30STRC" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'TODO'!$A$1:$F$2</definedName>
@@ -1527,7 +1528,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:N7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1687,6 +1688,134 @@
           <t>NODE_S1948_49_0002</t>
         </is>
       </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>NODE_S1948_49_0004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>30_Středočeská divize</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>league</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>L20</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>REG_STC</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>2-1-0</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>NODE_S1948_49_0005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>30_Středočeská divize Skupina A</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>group</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>L20</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>REG_STC</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>NODE_S1948_49_0004</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>2-1-0</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>NODE_S1948_49_0006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>30_Středočeská divize Skupina B</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>group</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>L20</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>REG_STC</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>NODE_S1948_49_0004</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>2-1-0</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1699,7 +1828,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J13"/>
+  <dimension ref="A1:J27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1767,7 +1896,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>LTC Praha [M]</t>
+          <t>JTO Sokol Pražský (LTC Praha)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -1814,7 +1943,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>ŠK Bratislava</t>
+          <t>ZJ Sokol NV Bratislava</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -1893,7 +2022,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>AC Stadion České Budějovice</t>
+          <t>JTO Sokol Stadion České Budějovice</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -1935,7 +2064,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Sokol Zbrojovka Židenice</t>
+          <t>ZSJ Zbrojovka Brno-Židenice</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1977,7 +2106,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>AC Sparta Bubeneč</t>
+          <t>JTO Sokol Sparta Bubeneč</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -2019,7 +2148,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Sokol Prostějov</t>
+          <t>JTO Sokol II Prostějov</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -2061,7 +2190,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>I. ČLTK Praha</t>
+          <t>JTO Sokol I Praha (I. ČLTK Praha)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -2235,6 +2364,566 @@
       <c r="J13" t="inlineStr">
         <is>
           <t>Pardubice</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>CLUB_S1948_49_0013</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Sokol Černošice</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>JTO Sokol Černošice</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>30STRC</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>L20</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Středočeská divize (PDF). prev_club_id zatím prázdný.</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Černošice</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>CLUB_S1948_49_0014</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Sokol Záběhlice-Zbraslav</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>JTO Sokol Záběhlice-Zbraslav</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>30STRC</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>L20</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Středočeská divize (PDF). prev_club_id zatím prázdný.</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Praha</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>CLUB_S1948_49_0015</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Sokol Slavia Praha</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>JTO Sokol Slavia Praha</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>30STRC</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>L20</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Středočeská divize (PDF). prev_club_id zatím prázdný.</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Praha</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>CLUB_S1948_49_0016</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Sokol Libeň</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>JTO Sokol Libeň</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>30STRC</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>L20</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Středočeská divize (PDF). prev_club_id zatím prázdný.</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Praha</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>CLUB_S1948_49_0017</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Sokol Roudnice nad Labem</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>JTO Sokol Roudnice nad Labem</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>30STRC</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>L20</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Středočeská divize (PDF). prev_club_id zatím prázdný.</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Roudnice nad Labem</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>CLUB_S1948_49_0018</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Sokol Kročehlavy</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>JTO Sokol Kročehlavy</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>30STRC</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>L20</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Středočeská divize (PDF). prev_club_id zatím prázdný.</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Kladno</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>CLUB_S1948_49_0019</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Sokol II Smíchov</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>JTO Sokol II Smíchov</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>30STRC</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>L20</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Středočeská divize (PDF). prev_club_id zatím prázdný.</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Praha</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>CLUB_S1948_49_0020</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Sokol Hostivař</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>JTO Sokol Hostivař</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>30STRC</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>L20</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Středočeská divize (PDF). prev_club_id zatím prázdný.</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Praha</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>CLUB_S1948_49_0021</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>ZSJ Kara Starý Kolín</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>ZSJ Kara Starý Kolín</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>30STRC</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>L20</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Středočeská divize (PDF). prev_club_id zatím prázdný.</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Starý Kolín</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>CLUB_S1948_49_0022</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Sokol Říčany</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>JTO Sokol Říčany</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>30STRC</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>L20</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Středočeská divize (PDF). prev_club_id zatím prázdný.</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Říčany</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>CLUB_S1948_49_0023</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Sokol Velké Popovice</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>JTO Sokol Velké Popovice</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>30STRC</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>L20</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Středočeská divize (PDF). prev_club_id zatím prázdný.</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Velké Popovice</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>CLUB_S1948_49_0024</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Sokol Modrobílí Kolín</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>JTO Sokol Modrobílí Kolín</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>30STRC</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>L20</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Středočeská divize (PDF). prev_club_id zatím prázdný.</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Kolín</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>CLUB_S1948_49_0025</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Sokol Vršovice-Bohemians</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>JTO Sokol Vršovice-Bohemians</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>30STRC</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>L20</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Středočeská divize (PDF). prev_club_id zatím prázdný.</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>Praha</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>CLUB_S1948_49_0026</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Sokol Čelákovice</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>JTO Sokol Čelákovice</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>30STRC</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>L20</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Středočeská divize (PDF). prev_club_id zatím prázdný.</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>Čelákovice</t>
         </is>
       </c>
     </row>
@@ -2315,7 +3004,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:A6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2328,14 +3017,35 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Republiková úroveň (extraliga + kvalifikace o ligu) zpracována z Wikipedie (en).</t>
+          <t>Nejvyšší soutěž (Státní liga) i divize zpracovány z PDF (dobový tisk).</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Krajské a okresní soutěže 1948/49 ZATÍM NEZPRACOVÁNY — Wiki nepokrývá regiony, čeká na podklady.</t>
+          <t>31. 3. 1948 sjednocení všech tělovýchovných organizací pod JTO Sokol — odtud sokolské názvy klubů (raw_name).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>3. 11. 1948: sloučení JTO Sokol Horácká Slavia Třebíč se ZSJ Zbrojovka Brno-Židenice; nový klub pod hlavičkou Zbrojovky převzal hráče i práva na Státní ligu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>9. 11. 1948: po odchodu všech hráčů ze Stadionu Podolí (do Sparty a I. ČLTK) klub vyřazen ze soutěže — JTO Sokol Stadion Podolí ukončil činnost.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Pražské oddíly (LTC, ATK, Sparta, I. ČLTK) hrály doma na ZS Štvanice; Prostějov v Olomouci; Židenice na ZS Za Lužánkami.</t>
         </is>
       </c>
     </row>
@@ -2421,7 +3131,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Wikipedia (en) — 1948-49 Czechoslovak Extraliga season</t>
+          <t>PDF sources/CZE1 + CZE2_3_nizsi (dobový tisk)</t>
         </is>
       </c>
     </row>
@@ -2481,7 +3191,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Šestý ročník. HC Stadion Podolí vyškrtnut (rozpad), nahrazen ATK Praha. Sokol Zbrojovka Židenice = sloučení Horácká Slavia Třebíč + Zbrojovka Židenice. I. ČLTK (finalista 1947/48) prohrál vše, 0 bodů.</t>
+          <t>Šestý ročník Státní ligy, 8 týmů jednokolově (mistr LTC Praha). Sokolské názvy (31.3.1948 sjednocení pod JTO Sokol). Stadion Podolí vyřazen 9.11.1948. Divize zpracovány po krajích.</t>
         </is>
       </c>
     </row>
@@ -2575,4 +3285,1264 @@
   <autoFilter ref="A1:F2"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:W17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="5" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="5" customWidth="1" min="5" max="5"/>
+    <col width="4" customWidth="1" min="6" max="6"/>
+    <col width="4" customWidth="1" min="7" max="7"/>
+    <col width="4" customWidth="1" min="8" max="8"/>
+    <col width="4" customWidth="1" min="9" max="9"/>
+    <col width="5" customWidth="1" min="10" max="10"/>
+    <col width="3" customWidth="1" min="11" max="11"/>
+    <col width="5" customWidth="1" min="12" max="12"/>
+    <col width="5" customWidth="1" min="13" max="13"/>
+    <col width="30" customWidth="1" min="14" max="14"/>
+    <col width="20" customWidth="1" min="15" max="15"/>
+    <col width="6" customWidth="1" min="16" max="16"/>
+    <col width="20" customWidth="1" min="17" max="17"/>
+    <col width="20" customWidth="1" min="18" max="18"/>
+    <col width="18" customWidth="1" min="19" max="19"/>
+    <col width="12" customWidth="1" min="20" max="20"/>
+    <col width="12" customWidth="1" min="21" max="21"/>
+    <col width="18" customWidth="1" min="22" max="22"/>
+    <col width="12" customWidth="1" min="23" max="23"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>row_type</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>block_name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>pos</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>club_name</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>GP</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>GF</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>GA</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>PTS</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>comp_path</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>node_id</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>level</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>club_id</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>prev_club_id</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>dest_node_id</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>dest_type</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>season_fate</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>tr_id</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>district</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Středočeská divize / Skupina A</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>NODE_S1948_49_0005</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>L20</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr"/>
+      <c r="T2" t="inlineStr"/>
+      <c r="U2" t="inlineStr"/>
+      <c r="V2" t="inlineStr"/>
+      <c r="W2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr"/>
+      <c r="C3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Sokol Černošice</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="n">
+        <v>6</v>
+      </c>
+      <c r="G3" t="n">
+        <v>5</v>
+      </c>
+      <c r="H3" t="n">
+        <v>1</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" t="n">
+        <v>39</v>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="L3" t="n">
+        <v>25</v>
+      </c>
+      <c r="M3" t="n">
+        <v>11</v>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Středočeská divize / Skupina A</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>NODE_S1948_49_0005</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>L20</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>CLUB_S1948_49_0013</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr"/>
+      <c r="T3" t="inlineStr"/>
+      <c r="U3" t="inlineStr"/>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>TR_S1948_49_00101</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr"/>
+      <c r="C4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Sokol Záběhlice-Zbraslav</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="n">
+        <v>6</v>
+      </c>
+      <c r="G4" t="n">
+        <v>4</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="n">
+        <v>2</v>
+      </c>
+      <c r="J4" t="n">
+        <v>27</v>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="L4" t="n">
+        <v>19</v>
+      </c>
+      <c r="M4" t="n">
+        <v>8</v>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Středočeská divize / Skupina A</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>NODE_S1948_49_0005</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>L20</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>CLUB_S1948_49_0014</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr"/>
+      <c r="S4" t="inlineStr"/>
+      <c r="T4" t="inlineStr"/>
+      <c r="U4" t="inlineStr"/>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>TR_S1948_49_00102</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr"/>
+      <c r="C5" t="n">
+        <v>3</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Sokol Slavia Praha</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="n">
+        <v>6</v>
+      </c>
+      <c r="G5" t="n">
+        <v>3</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="n">
+        <v>3</v>
+      </c>
+      <c r="J5" t="n">
+        <v>26</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="L5" t="n">
+        <v>18</v>
+      </c>
+      <c r="M5" t="n">
+        <v>6</v>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Středočeská divize / Skupina A</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>NODE_S1948_49_0005</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>L20</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>CLUB_S1948_49_0015</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr"/>
+      <c r="S5" t="inlineStr"/>
+      <c r="T5" t="inlineStr"/>
+      <c r="U5" t="inlineStr"/>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>TR_S1948_49_00103</t>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr"/>
+      <c r="C6" t="n">
+        <v>4</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Sokol Libeň</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="n">
+        <v>6</v>
+      </c>
+      <c r="G6" t="n">
+        <v>3</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="n">
+        <v>3</v>
+      </c>
+      <c r="J6" t="n">
+        <v>25</v>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="L6" t="n">
+        <v>28</v>
+      </c>
+      <c r="M6" t="n">
+        <v>6</v>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Středočeská divize / Skupina A</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>NODE_S1948_49_0005</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>L20</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>CLUB_S1948_49_0016</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr"/>
+      <c r="S6" t="inlineStr"/>
+      <c r="T6" t="inlineStr"/>
+      <c r="U6" t="inlineStr"/>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>TR_S1948_49_00104</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="n">
+        <v>5</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Sokol Roudnice nad Labem</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="n">
+        <v>6</v>
+      </c>
+      <c r="G7" t="n">
+        <v>3</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" t="n">
+        <v>3</v>
+      </c>
+      <c r="J7" t="n">
+        <v>18</v>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="L7" t="n">
+        <v>23</v>
+      </c>
+      <c r="M7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Středočeská divize / Skupina A</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>NODE_S1948_49_0005</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>L20</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>CLUB_S1948_49_0017</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr"/>
+      <c r="S7" t="inlineStr"/>
+      <c r="T7" t="inlineStr"/>
+      <c r="U7" t="inlineStr"/>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>TR_S1948_49_00105</t>
+        </is>
+      </c>
+      <c r="W7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="n">
+        <v>6</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Sokol Kročehlavy</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="n">
+        <v>6</v>
+      </c>
+      <c r="G8" t="n">
+        <v>2</v>
+      </c>
+      <c r="H8" t="n">
+        <v>1</v>
+      </c>
+      <c r="I8" t="n">
+        <v>3</v>
+      </c>
+      <c r="J8" t="n">
+        <v>24</v>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="L8" t="n">
+        <v>18</v>
+      </c>
+      <c r="M8" t="n">
+        <v>5</v>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Středočeská divize / Skupina A</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>NODE_S1948_49_0005</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>L20</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>CLUB_S1948_49_0018</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr"/>
+      <c r="S8" t="inlineStr"/>
+      <c r="T8" t="inlineStr"/>
+      <c r="U8" t="inlineStr"/>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>TR_S1948_49_00106</t>
+        </is>
+      </c>
+      <c r="W8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="n">
+        <v>7</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Sokol II Smíchov</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="n">
+        <v>6</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" t="n">
+        <v>6</v>
+      </c>
+      <c r="J9" t="n">
+        <v>15</v>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="L9" t="n">
+        <v>43</v>
+      </c>
+      <c r="M9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Středočeská divize / Skupina A</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>NODE_S1948_49_0005</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>L20</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>CLUB_S1948_49_0019</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr"/>
+      <c r="S9" t="inlineStr"/>
+      <c r="T9" t="inlineStr"/>
+      <c r="U9" t="inlineStr"/>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>TR_S1948_49_00107</t>
+        </is>
+      </c>
+      <c r="W9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Středočeská divize / Skupina B</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>NODE_S1948_49_0006</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>L20</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr"/>
+      <c r="R10" t="inlineStr"/>
+      <c r="S10" t="inlineStr"/>
+      <c r="T10" t="inlineStr"/>
+      <c r="U10" t="inlineStr"/>
+      <c r="V10" t="inlineStr"/>
+      <c r="W10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Sokol Hostivař</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="n">
+        <v>6</v>
+      </c>
+      <c r="G11" t="n">
+        <v>6</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" t="n">
+        <v>67</v>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="L11" t="n">
+        <v>22</v>
+      </c>
+      <c r="M11" t="n">
+        <v>12</v>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>Středočeská divize / Skupina B</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>NODE_S1948_49_0006</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>L20</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>CLUB_S1948_49_0020</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr"/>
+      <c r="S11" t="inlineStr"/>
+      <c r="T11" t="inlineStr"/>
+      <c r="U11" t="inlineStr"/>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>TR_S1948_49_00108</t>
+        </is>
+      </c>
+      <c r="W11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr"/>
+      <c r="C12" t="n">
+        <v>2</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>ZSJ Kara Starý Kolín</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="n">
+        <v>6</v>
+      </c>
+      <c r="G12" t="n">
+        <v>5</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" t="n">
+        <v>1</v>
+      </c>
+      <c r="J12" t="n">
+        <v>53</v>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="L12" t="n">
+        <v>28</v>
+      </c>
+      <c r="M12" t="n">
+        <v>10</v>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>Středočeská divize / Skupina B</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>NODE_S1948_49_0006</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>L20</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>CLUB_S1948_49_0021</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr"/>
+      <c r="S12" t="inlineStr"/>
+      <c r="T12" t="inlineStr"/>
+      <c r="U12" t="inlineStr"/>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>TR_S1948_49_00109</t>
+        </is>
+      </c>
+      <c r="W12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr"/>
+      <c r="C13" t="n">
+        <v>3</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Sokol Říčany</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="n">
+        <v>6</v>
+      </c>
+      <c r="G13" t="n">
+        <v>4</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" t="n">
+        <v>2</v>
+      </c>
+      <c r="J13" t="n">
+        <v>37</v>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="L13" t="n">
+        <v>41</v>
+      </c>
+      <c r="M13" t="n">
+        <v>8</v>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>Středočeská divize / Skupina B</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>NODE_S1948_49_0006</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>L20</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>CLUB_S1948_49_0022</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr"/>
+      <c r="S13" t="inlineStr"/>
+      <c r="T13" t="inlineStr"/>
+      <c r="U13" t="inlineStr"/>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>TR_S1948_49_00110</t>
+        </is>
+      </c>
+      <c r="W13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr"/>
+      <c r="C14" t="n">
+        <v>4</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Sokol Velké Popovice</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="n">
+        <v>6</v>
+      </c>
+      <c r="G14" t="n">
+        <v>3</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" t="n">
+        <v>3</v>
+      </c>
+      <c r="J14" t="n">
+        <v>37</v>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="L14" t="n">
+        <v>38</v>
+      </c>
+      <c r="M14" t="n">
+        <v>6</v>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>Středočeská divize / Skupina B</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>NODE_S1948_49_0006</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>L20</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>CLUB_S1948_49_0023</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr"/>
+      <c r="S14" t="inlineStr"/>
+      <c r="T14" t="inlineStr"/>
+      <c r="U14" t="inlineStr"/>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>TR_S1948_49_00111</t>
+        </is>
+      </c>
+      <c r="W14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr"/>
+      <c r="C15" t="n">
+        <v>5</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Sokol Modrobílí Kolín</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="n">
+        <v>6</v>
+      </c>
+      <c r="G15" t="n">
+        <v>2</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" t="n">
+        <v>4</v>
+      </c>
+      <c r="J15" t="n">
+        <v>40</v>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="L15" t="n">
+        <v>39</v>
+      </c>
+      <c r="M15" t="n">
+        <v>4</v>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>Středočeská divize / Skupina B</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>NODE_S1948_49_0006</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>L20</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>CLUB_S1948_49_0024</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr"/>
+      <c r="S15" t="inlineStr"/>
+      <c r="T15" t="inlineStr"/>
+      <c r="U15" t="inlineStr"/>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>TR_S1948_49_00112</t>
+        </is>
+      </c>
+      <c r="W15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr"/>
+      <c r="C16" t="n">
+        <v>6</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Sokol Vršovice-Bohemians</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="n">
+        <v>6</v>
+      </c>
+      <c r="G16" t="n">
+        <v>1</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" t="n">
+        <v>5</v>
+      </c>
+      <c r="J16" t="n">
+        <v>33</v>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="L16" t="n">
+        <v>43</v>
+      </c>
+      <c r="M16" t="n">
+        <v>2</v>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>Středočeská divize / Skupina B</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>NODE_S1948_49_0006</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>L20</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>CLUB_S1948_49_0025</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr"/>
+      <c r="S16" t="inlineStr"/>
+      <c r="T16" t="inlineStr"/>
+      <c r="U16" t="inlineStr"/>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>TR_S1948_49_00113</t>
+        </is>
+      </c>
+      <c r="W16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr"/>
+      <c r="C17" t="n">
+        <v>7</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Sokol Čelákovice</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="n">
+        <v>6</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" t="n">
+        <v>6</v>
+      </c>
+      <c r="J17" t="n">
+        <v>22</v>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="L17" t="n">
+        <v>78</v>
+      </c>
+      <c r="M17" t="n">
+        <v>0</v>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>Středočeská divize / Skupina B</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>NODE_S1948_49_0006</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>L20</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>CLUB_S1948_49_0026</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr"/>
+      <c r="S17" t="inlineStr"/>
+      <c r="T17" t="inlineStr"/>
+      <c r="U17" t="inlineStr"/>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>TR_S1948_49_00114</t>
+        </is>
+      </c>
+      <c r="W17" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Lektorování 48/49 župní: audit konzistence (3 flagy do TODO)
Kontrola V+R+P=GP a body=2·V+R + duplicity + artefakty napříč 15 župami:
import čistý (560 týmů), nalezeny 3 překlepy ve zdroji (Dobrovice, H.Slavia
Třebíč, Podvesná) → zaznamenány do TODO k budoucímu ověření z archivu, neopravují
se naslepo.

https://claude.ai/code/session_01BhRGgVD2Sevo7xfvYw5ngZ
</commit_message>
<xml_diff>
--- a/data/S1948_49_FINAL.xlsx
+++ b/data/S1948_49_FINAL.xlsx
@@ -4004,7 +4004,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4048,9 +4048,77 @@
       </c>
     </row>
     <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>lektor</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>ZSEVC II.tř.A/sk.C · Sokol Dobrovice</t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>(žádné otevřené položky — sezóna OK)</t>
+          <t>Nesedí rozpis: GP=5, ale V+R+P=4 (1 zápas chybí). Ověřit z archivu/tisku.</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>ne</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>lektor</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>ZHORA II.tř./sk.C · Sokol Horácká Slavia Třebíč</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Body=2 při 2 výhrách (má být 4?). Překlep ve zdroji – ověřit.</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>ne</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>lektor</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>ZHANA I.tř./sk.B · SK Podvesná</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Body=10 při 4 výhrách (2-1-0 → 8). Nesedí V nebo body – ověřit.</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>ne</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Blbuvzdorné názvy: přepis kódů na plné názvy v 73 sezónách (expand_names.py) + desktop strom jako hierarchie (org chart) s plnými názvy
</commit_message>
<xml_diff>
--- a/data/S1948_49_FINAL.xlsx
+++ b/data/S1948_49_FINAL.xlsx
@@ -18719,7 +18719,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>30_Středočeská divize</t>
+          <t>Středočeská divize</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -18751,7 +18751,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>30_Středočeská divize Skupina A</t>
+          <t>Středočeská divize Skupina A</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -18788,7 +18788,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>30_Středočeská divize Skupina B</t>
+          <t>Středočeská divize Skupina B</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -18825,7 +18825,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>30_Západočeská divize</t>
+          <t>Západočeská divize</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -18857,7 +18857,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>30_Západočeská Skupina A</t>
+          <t>Západočeská Skupina A</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -18894,7 +18894,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>30_Západočeská Skupina B</t>
+          <t>Západočeská Skupina B</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -18931,7 +18931,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>30_Východočeská divize</t>
+          <t>Východočeská divize</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -18963,7 +18963,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>30_Východočeská Skupina A</t>
+          <t>Východočeská Skupina A</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -19000,7 +19000,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>30_Východočeská Skupina B</t>
+          <t>Východočeská Skupina B</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -19037,7 +19037,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>30_Moravskoslezská divize</t>
+          <t>Moravskoslezská divize</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -19069,7 +19069,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>30_Moravskoslezská Skupina A</t>
+          <t>Moravskoslezská Skupina A</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -19106,7 +19106,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>30_Moravskoslezská Skupina B</t>
+          <t>Moravskoslezská Skupina B</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -19143,7 +19143,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>30_Slovenská oblastná liga divize</t>
+          <t>Slovenská oblastná liga divize</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -19175,7 +19175,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>30_Slovenská oblastná liga Skupina západ</t>
+          <t>Slovenská oblastná liga Skupina západ</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -19212,7 +19212,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>30_Slovenská oblastná liga Skupina východ</t>
+          <t>Slovenská oblastná liga Skupina východ</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">

</xml_diff>

<commit_message>
DB osudy podle fází: postup/sestup už ne ze základní části — fázové štítky (play off / o udržení / o umístění / kvalifikace / prolínací) z feeds_into(_loser)+členství; skupina o udržení: udržel se vs sestup; 1915 oprav v 71 sezónách + report k ruční revizi (fix_fates.py)
</commit_message>
<xml_diff>
--- a/data/S1948_49_FINAL.xlsx
+++ b/data/S1948_49_FINAL.xlsx
@@ -3292,6 +3292,11 @@
           <t>CLUB_S1948_49_0033</t>
         </is>
       </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>play off</t>
+        </is>
+      </c>
       <c r="V3" t="inlineStr">
         <is>
           <t>TR_S1948_49_00248</t>
@@ -3356,6 +3361,11 @@
       <c r="Q4" t="inlineStr">
         <is>
           <t>CLUB_S1948_49_0040</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>play off</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">

</xml_diff>